<commit_message>
feat: update Colombia Perfect Store scoring
</commit_message>
<xml_diff>
--- a/base_prov_co/cruz_verde/cruz_verde_abbott_2026_09_16.xlsx
+++ b/base_prov_co/cruz_verde/cruz_verde_abbott_2026_09_16.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,55 +451,60 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>MARCA</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>seller</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ventas</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>valoracion</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>reviews</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>img_count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>video_count</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>title_count_characters</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>count_character_desc</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>url_producto</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>disponibilidad</t>
         </is>
@@ -526,43 +531,46 @@
           <t>8427030008608</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENSURE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Abbott</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>5</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>53</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>https://www.cruzverde.com.co/ensure-advance-vainilla-con-proteina--hmb-polvo-850g/COCV_129816.html</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>DISPONIBLE</t>
         </is>

</xml_diff>